<commit_message>
z roll and pitch
</commit_message>
<xml_diff>
--- a/velocity/sheets/velocities_table.xlsx
+++ b/velocity/sheets/velocities_table.xlsx
@@ -8,19 +8,32 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ishayu/Documents/GitHub/ishayu_metrics/velocity/sheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{4F920E7E-FBE8-4348-B00B-44190D14C9D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D5AB975-3A14-D949-97D2-D35326A31398}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3260" yWindow="2160" windowWidth="28040" windowHeight="17440" xr2:uid="{E1A3D8A8-AEDA-3441-B949-BD213C392CE8}"/>
   </bookViews>
   <sheets>
     <sheet name="velocities_table" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>Terrain</t>
   </si>
@@ -83,6 +96,9 @@
   </si>
   <si>
     <t>Faster than predefined?</t>
+  </si>
+  <si>
+    <t>Amount faster than predefined</t>
   </si>
 </sst>
 </file>
@@ -581,7 +597,7 @@
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
@@ -959,7 +975,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69115A4A-68EB-1E45-88F5-11975D390585}">
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24.5" bestFit="1" customWidth="1"/>
@@ -971,7 +987,7 @@
     <col min="8" max="8" width="14.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -999,8 +1015,11 @@
       <c r="I1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -1021,7 +1040,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1032,7 +1051,7 @@
         <v>20.186580125534999</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1062,8 +1081,12 @@
         <f>E4&lt;0.05</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J4">
+        <f>B5-B4</f>
+        <v>61.029971337755697</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -1074,7 +1097,7 @@
         <v>19.6572158034054</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -1100,8 +1123,12 @@
         <f>E6&lt;0.05</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J6">
+        <f>B7-B6</f>
+        <v>23.472831299941902</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -1112,7 +1139,7 @@
         <v>19.6172847508725</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -1142,8 +1169,12 @@
         <f>E8&lt;0.05</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J8">
+        <f>B9-B8</f>
+        <v>9.4710353456432017</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -1154,7 +1185,7 @@
         <v>10.2520324176818</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>15</v>
       </c>
@@ -1184,8 +1215,12 @@
         <f>E10&lt;0.05</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J10">
+        <f>B11-B10</f>
+        <v>25.009133358552901</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -1196,7 +1231,7 @@
         <v>9.79511576599897</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>17</v>
       </c>
@@ -1226,8 +1261,12 @@
         <f>E12&lt;0.05</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J12">
+        <f>B13-B12</f>
+        <v>37.430014779007607</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>18</v>
       </c>
@@ -1236,6 +1275,12 @@
       </c>
       <c r="C13" s="2">
         <v>16.177894032288702</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J14">
+        <f>AVERAGE(J4,J6,J8,J10,J12)</f>
+        <v>31.282597224180261</v>
       </c>
     </row>
   </sheetData>

</xml_diff>